<commit_message>
Added Rate files for waste management/Battery collection process (refurb 0 temporarily); modified config files to read in rate files; modified main script (EV_model.ipynb) to have the proper flows and processes for the waste management/Battery collection process
</commit_message>
<xml_diff>
--- a/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model.xlsx
+++ b/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\EV_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DE979C-A3D6-43A4-82B5-5A7451D751C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903FD400-0D50-4E6B-8747-AA3FB14FF215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="145">
   <si>
     <t>Description</t>
   </si>
@@ -417,9 +417,6 @@
     <t>ODYM_Tutorial6_EVConsumptionLL</t>
   </si>
   <si>
-    <t>ODYM_Tutorial6_EVLIB</t>
-  </si>
-  <si>
     <t>Final consumption of EVs, exogenous model driver</t>
   </si>
   <si>
@@ -430,6 +427,48 @@
   </si>
   <si>
     <t>[3]</t>
+  </si>
+  <si>
+    <t>ODYM_T6_ToUsedExportRateLL</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e6</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e7</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e8</t>
+  </si>
+  <si>
+    <t>6213e899-8367-483a-8d09-a0c0831c22e9</t>
+  </si>
+  <si>
+    <t>ODYM_T6_ToLandfillRateLL</t>
+  </si>
+  <si>
+    <t>Share of flow after use going to landfill. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>Share of flow after use going to used export. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>Share of flow after use going to refurbishment. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>Share of flow after use going to recycling. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>ODYM_T6_ToRefurbishmentRateLL</t>
+  </si>
+  <si>
+    <t>ODYM_T6_ToRecyclingRateLL</t>
+  </si>
+  <si>
+    <t>ODYM_Tutorial6_EV_Model</t>
+  </si>
+  <si>
+    <t>Refurbishing</t>
   </si>
 </sst>
 </file>
@@ -637,7 +676,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -718,6 +757,8 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1182,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J60"/>
+  <dimension ref="B2:J65"/>
   <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4.77734375" customWidth="1"/>
@@ -1223,7 +1264,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
@@ -1402,7 +1443,7 @@
         <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>24</v>
@@ -1680,104 +1721,92 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E37" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B39" s="18" t="s">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C38" s="31">
+        <v>10</v>
+      </c>
+      <c r="D38" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B40" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="20"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C40" s="26" t="s">
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="20"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C41" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D40" s="23" t="s">
+      <c r="D41" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="E41" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F41" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="G40" s="39" t="s">
+      <c r="G41" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="H40" s="23" t="s">
+      <c r="H41" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="I40" s="36" t="s">
+      <c r="I41" s="36" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C41" t="s">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C42" t="s">
         <v>117</v>
       </c>
-      <c r="D41" s="38" t="s">
+      <c r="D42" s="38" t="s">
         <v>124</v>
-      </c>
-      <c r="E41" t="s">
-        <v>97</v>
-      </c>
-      <c r="F41" t="s">
-        <v>64</v>
-      </c>
-      <c r="G41" t="s">
-        <v>31</v>
-      </c>
-      <c r="H41" t="s">
-        <v>31</v>
-      </c>
-      <c r="I41" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C42" s="27" t="s">
-        <v>126</v>
-      </c>
-      <c r="D42" t="s">
-        <v>128</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
       </c>
       <c r="F42" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="G42" t="s">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="H42" t="s">
         <v>31</v>
       </c>
       <c r="I42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D43" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E43" t="s">
         <v>97</v>
       </c>
       <c r="F43" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G43" t="s">
         <v>81</v>
@@ -1785,16 +1814,16 @@
       <c r="H43" t="s">
         <v>31</v>
       </c>
-      <c r="I43" s="37" t="s">
-        <v>100</v>
+      <c r="I43" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D44" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="E44" t="s">
         <v>97</v>
@@ -1809,41 +1838,44 @@
         <v>31</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D45" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E45" t="s">
         <v>97</v>
       </c>
       <c r="F45" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G45" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="H45" t="s">
         <v>31</v>
       </c>
       <c r="I45" s="37" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C46" s="27" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="D46" t="s">
+        <v>108</v>
       </c>
       <c r="E46" t="s">
         <v>97</v>
       </c>
       <c r="F46" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G46" t="s">
         <v>86</v>
@@ -1852,80 +1884,192 @@
         <v>31</v>
       </c>
       <c r="I46" s="37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C47" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="E47" t="s">
+        <v>97</v>
+      </c>
+      <c r="F47" t="s">
+        <v>110</v>
+      </c>
+      <c r="G47" t="s">
+        <v>86</v>
+      </c>
+      <c r="H47" t="s">
+        <v>31</v>
+      </c>
+      <c r="I47" s="37" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C47" s="27"/>
-    </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B48" s="18" t="s">
+      <c r="C48" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="D48" t="s">
+        <v>137</v>
+      </c>
+      <c r="E48" t="s">
+        <v>97</v>
+      </c>
+      <c r="F48" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="G48" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="H48" t="s">
+        <v>31</v>
+      </c>
+      <c r="I48" s="41" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C49" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="D49" t="s">
+        <v>138</v>
+      </c>
+      <c r="E49" t="s">
+        <v>97</v>
+      </c>
+      <c r="F49" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="G49" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="H49" t="s">
+        <v>31</v>
+      </c>
+      <c r="I49" s="41" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C50" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="D50" t="s">
+        <v>139</v>
+      </c>
+      <c r="E50" t="s">
+        <v>97</v>
+      </c>
+      <c r="F50" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="G50" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="H50" t="s">
+        <v>31</v>
+      </c>
+      <c r="I50" s="41" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C51" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="D51" t="s">
+        <v>140</v>
+      </c>
+      <c r="E51" t="s">
+        <v>97</v>
+      </c>
+      <c r="F51" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="G51" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="H51" t="s">
+        <v>31</v>
+      </c>
+      <c r="I51" s="41" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C52" s="27"/>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B53" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
-      <c r="E48" s="19"/>
-      <c r="F48" s="19"/>
-      <c r="G48" s="19"/>
-      <c r="H48" s="20"/>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C49" t="s">
+      <c r="C53" s="19"/>
+      <c r="D53" s="19"/>
+      <c r="E53" s="19"/>
+      <c r="F53" s="19"/>
+      <c r="G53" s="19"/>
+      <c r="H53" s="20"/>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C54" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C50" s="27" t="s">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C55" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="D50" s="33" t="s">
+      <c r="D55" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E55" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D51" s="33"/>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D52" s="33"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D53" s="33"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D54" s="33"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D55" s="33"/>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B57" s="18" t="s">
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D56" s="33"/>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D57" s="33"/>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D58" s="33"/>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D59" s="33"/>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="D60" s="33"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B62" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="20"/>
-    </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C58" t="s">
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="20"/>
+    </row>
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C63" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B60" s="18" t="s">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B65" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="20"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changes to add a working refurbishment process. Refer to list of changes in the first chunk of the .ipynb file under 2025-07-21
</commit_message>
<xml_diff>
--- a/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model.xlsx
+++ b/docs/Files/EV_model/ODYM_Config_Tutorial6_EV_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvend\Documents\CodeProjects\ODYM\docs\Files\EV_model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903FD400-0D50-4E6B-8747-AA3FB14FF215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2138F74B-B3C0-47C0-A7FE-8D77CD6C3300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="844" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,9 +336,6 @@
     <t>6738f872-8ec9-4ba5-986b-6da947f03289</t>
   </si>
   <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e5</t>
-  </si>
-  <si>
     <t>Sgmw</t>
   </si>
   <si>
@@ -360,9 +357,6 @@
     <t>Swm</t>
   </si>
   <si>
-    <t>Share of input scrap that is recovered as secondary material</t>
-  </si>
-  <si>
     <t>a3e33053-ab7a-4979-be82-d14c6e5eecef</t>
   </si>
   <si>
@@ -390,9 +384,6 @@
     <t>ODYM_Tutorial6_LifetimeLL</t>
   </si>
   <si>
-    <t>ODYM_Tutorial6_EoLRecoveryRateLL</t>
-  </si>
-  <si>
     <t>ODYM_Tutorial6_FabricationYieldLossLL</t>
   </si>
   <si>
@@ -420,9 +411,6 @@
     <t>Final consumption of EVs, exogenous model driver</t>
   </si>
   <si>
-    <t>EoL recovery rate of scrap batteries from products</t>
-  </si>
-  <si>
     <t>Landfill</t>
   </si>
   <si>
@@ -438,9 +426,6 @@
     <t>6213e899-8367-483a-8d09-a0c0831c22e7</t>
   </si>
   <si>
-    <t>6213e899-8367-483a-8d09-a0c0831c22e8</t>
-  </si>
-  <si>
     <t>6213e899-8367-483a-8d09-a0c0831c22e9</t>
   </si>
   <si>
@@ -453,22 +438,37 @@
     <t>Share of flow after use going to used export. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
   </si>
   <si>
-    <t>Share of flow after use going to refurbishment. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
-  </si>
-  <si>
     <t>Share of flow after use going to recycling. Index structure and Aspect order match based on EolRecovery rate as these rates share the same process.</t>
   </si>
   <si>
-    <t>ODYM_T6_ToRefurbishmentRateLL</t>
-  </si>
-  <si>
     <t>ODYM_T6_ToRecyclingRateLL</t>
   </si>
   <si>
     <t>ODYM_Tutorial6_EV_Model</t>
   </si>
   <si>
-    <t>Refurbishing</t>
+    <t>ODYM_T6_ScrapToRefurbishmentRateLL</t>
+  </si>
+  <si>
+    <t>Share of scrap flow after use going to refurbishment. Index structure and Aspect order match based on RemeltingYield as these rates share the same process.</t>
+  </si>
+  <si>
+    <t>Share of input scrap that is recovered as secondary material and goes to recycling.</t>
+  </si>
+  <si>
+    <t>38ed7154-01c2-4d21-8128-df10bbd150a6</t>
+  </si>
+  <si>
+    <t>ODYM_T6_RefurbishmentSectorSplitLL</t>
+  </si>
+  <si>
+    <t>Distribution of goods after refurbishment. Based on ODYM_Tutorial6_SectorSplitLL</t>
+  </si>
+  <si>
+    <t>a3e33053-ab7a-4979-be82-d14c6e5eece1</t>
+  </si>
+  <si>
+    <t>Refurbishment</t>
   </si>
 </sst>
 </file>
@@ -548,7 +548,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -570,6 +570,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -676,7 +688,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -759,6 +771,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1077,7 +1094,7 @@
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G4" s="35"/>
     </row>
@@ -1264,7 +1281,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
@@ -1272,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
@@ -1319,7 +1336,7 @@
         <v>6</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J10" s="13"/>
     </row>
@@ -1397,7 +1414,7 @@
         <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H16" s="21" t="s">
         <v>23</v>
@@ -1420,7 +1437,7 @@
         <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H17" s="21" t="s">
         <v>78</v>
@@ -1443,7 +1460,7 @@
         <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H18" s="21" t="s">
         <v>24</v>
@@ -1486,7 +1503,7 @@
         <v>82</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G20" t="s">
         <v>89</v>
@@ -1644,7 +1661,7 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E30" t="s">
         <v>58</v>
@@ -1677,7 +1694,7 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E33" t="s">
         <v>57</v>
@@ -1688,7 +1705,7 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E34" t="s">
         <v>58</v>
@@ -1699,7 +1716,7 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E35" t="s">
         <v>57</v>
@@ -1721,7 +1738,7 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E37" t="s">
         <v>57</v>
@@ -1774,10 +1791,10 @@
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E42" t="s">
         <v>97</v>
@@ -1797,16 +1814,16 @@
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C43" s="27" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D43" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E43" t="s">
         <v>97</v>
       </c>
       <c r="F43" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G43" t="s">
         <v>81</v>
@@ -1820,16 +1837,16 @@
     </row>
     <row r="44" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C44" s="27" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D44" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="E44" t="s">
         <v>97</v>
       </c>
       <c r="F44" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G44" t="s">
         <v>81</v>
@@ -1838,87 +1855,88 @@
         <v>31</v>
       </c>
       <c r="I44" s="37" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C45" s="27" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D45" t="s">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="E45" t="s">
         <v>97</v>
       </c>
-      <c r="F45" t="s">
-        <v>101</v>
-      </c>
-      <c r="G45" t="s">
-        <v>81</v>
-      </c>
-      <c r="H45" t="s">
+      <c r="F45" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="H45" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="I45" s="37" t="s">
-        <v>104</v>
+      <c r="I45" s="43" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="46" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C46" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="C46" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="D46" s="45"/>
+      <c r="E46" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="F46" s="45" t="s">
         <v>108</v>
       </c>
-      <c r="E46" t="s">
-        <v>97</v>
-      </c>
-      <c r="F46" t="s">
+      <c r="G46" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="H46" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="I46" s="46" t="s">
         <v>107</v>
-      </c>
-      <c r="G46" t="s">
-        <v>86</v>
-      </c>
-      <c r="H46" t="s">
-        <v>31</v>
-      </c>
-      <c r="I46" s="37" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C47" s="27" t="s">
-        <v>121</v>
+        <v>131</v>
+      </c>
+      <c r="D47" t="s">
+        <v>132</v>
       </c>
       <c r="E47" t="s">
         <v>97</v>
       </c>
-      <c r="F47" t="s">
-        <v>110</v>
-      </c>
-      <c r="G47" t="s">
-        <v>86</v>
+      <c r="F47" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="G47" s="40" t="s">
+        <v>81</v>
       </c>
       <c r="H47" t="s">
         <v>31</v>
       </c>
-      <c r="I47" s="37" t="s">
-        <v>109</v>
+      <c r="I47" s="41" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C48" s="27" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="D48" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E48" t="s">
         <v>97</v>
       </c>
       <c r="F48" s="40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G48" s="40" t="s">
         <v>81</v>
@@ -1927,21 +1945,21 @@
         <v>31</v>
       </c>
       <c r="I48" s="41" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="49" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C49" s="27" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D49" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E49" t="s">
         <v>97</v>
       </c>
       <c r="F49" s="40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G49" s="40" t="s">
         <v>81</v>
@@ -1950,57 +1968,54 @@
         <v>31</v>
       </c>
       <c r="I49" s="41" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C50" s="27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D50" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E50" t="s">
         <v>97</v>
       </c>
-      <c r="F50" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="G50" s="40" t="s">
-        <v>81</v>
-      </c>
-      <c r="H50" t="s">
+      <c r="F50" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="G50" s="42" t="s">
+        <v>86</v>
+      </c>
+      <c r="H50" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="I50" s="41" t="s">
-        <v>134</v>
+      <c r="I50" s="43" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C51" s="27" t="s">
+      <c r="C51" s="44" t="s">
+        <v>141</v>
+      </c>
+      <c r="D51" s="45" t="s">
         <v>142</v>
       </c>
-      <c r="D51" t="s">
-        <v>140</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="E51" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="F51" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="G51" s="40" t="s">
-        <v>81</v>
-      </c>
-      <c r="H51" t="s">
+      <c r="F51" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G51" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="H51" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="I51" s="41" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C52" s="27"/>
+      <c r="I51" s="46" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B53" s="18" t="s">
@@ -2062,7 +2077,7 @@
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B65" s="18" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>

</xml_diff>